<commit_message>
auto: reporte semana 2026-08-03 → 2026-08-09
</commit_message>
<xml_diff>
--- a/latest-events.xlsx
+++ b/latest-events.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D140"/>
+  <dimension ref="A1:D138"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,7 +422,7 @@
         <v>6618</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-07-30 16:53:20</v>
+        <v>2026-08-03 09:54:04</v>
       </c>
       <c r="D2" t="str">
         <v>NO</v>
@@ -436,10 +436,10 @@
         <v>6618</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-07-30 16:53:20</v>
+        <v>2026-08-03 21:38:01</v>
       </c>
       <c r="D3" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="4">
@@ -450,21 +450,21 @@
         <v>6618</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-07-30 21:26:39</v>
+        <v>2026-08-04 17:17:29</v>
       </c>
       <c r="D4" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GC MAXUS PCRF-25 TERRENO</v>
+        <v>DONGFENG DF6 SRSR-97</v>
       </c>
       <c r="B5">
-        <v>6617</v>
+        <v>6618</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-07-31 12:39:58</v>
+        <v>2026-08-07 16:39:44</v>
       </c>
       <c r="D5" t="str">
         <v>NO</v>
@@ -472,13 +472,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B6">
-        <v>6616</v>
+        <v>6617</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-07-30 15:06:14</v>
+        <v>2026-08-03 07:42:06</v>
       </c>
       <c r="D6" t="str">
         <v>NO</v>
@@ -486,13 +486,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B7">
-        <v>6616</v>
+        <v>6617</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-07-30 15:06:14</v>
+        <v>2026-08-04 10:24:14</v>
       </c>
       <c r="D7" t="str">
         <v>NO</v>
@@ -500,41 +500,41 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B8">
-        <v>6616</v>
+        <v>6617</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-07-30 20:17:06</v>
+        <v>2026-08-04 16:37:27</v>
       </c>
       <c r="D8" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GC RXDL-59 OPERACIONES</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B9">
-        <v>6581</v>
+        <v>6617</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-07-27 09:07:04</v>
+        <v>2026-08-07 20:05:00</v>
       </c>
       <c r="D9" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GC RXDL-59 OPERACIONES</v>
+        <v>GC MAXUS PKFF-65 G VICENCIO</v>
       </c>
       <c r="B10">
-        <v>6581</v>
+        <v>6616</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-07-30 21:03:38</v>
+        <v>2026-08-04 20:29:03</v>
       </c>
       <c r="D10" t="str">
         <v>SI</v>
@@ -548,7 +548,7 @@
         <v>6608</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-07-30 14:38:45</v>
+        <v>2026-08-03 11:30:01</v>
       </c>
       <c r="D11" t="str">
         <v>NO</v>
@@ -562,10 +562,10 @@
         <v>6608</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-07-30 14:38:45</v>
+        <v>2026-08-03 22:05:36</v>
       </c>
       <c r="D12" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="13">
@@ -576,7 +576,7 @@
         <v>6608</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-07-30 14:47:35</v>
+        <v>2026-08-04 18:08:38</v>
       </c>
       <c r="D13" t="str">
         <v>NO</v>
@@ -590,7 +590,7 @@
         <v>6608</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-07-30 15:47:11</v>
+        <v>2026-08-07 16:24:51</v>
       </c>
       <c r="D14" t="str">
         <v>NO</v>
@@ -598,16 +598,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B15">
-        <v>6608</v>
+        <v>6609</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-07-30 20:43:05</v>
+        <v>2026-08-03 11:20:30</v>
       </c>
       <c r="D15" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="16">
@@ -618,10 +618,10 @@
         <v>6609</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-07-30 14:35:58</v>
+        <v>2026-08-03 21:25:32</v>
       </c>
       <c r="D16" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="17">
@@ -632,10 +632,10 @@
         <v>6609</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-07-30 14:35:58</v>
+        <v>2026-08-03 22:01:58</v>
       </c>
       <c r="D17" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="18">
@@ -646,7 +646,7 @@
         <v>6609</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-07-30 16:36:45</v>
+        <v>2026-08-04 16:37:54</v>
       </c>
       <c r="D18" t="str">
         <v>NO</v>
@@ -660,7 +660,7 @@
         <v>6609</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-07-30 16:36:45</v>
+        <v>2026-08-07 15:22:06</v>
       </c>
       <c r="D19" t="str">
         <v>NO</v>
@@ -668,27 +668,27 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B20">
-        <v>6609</v>
+        <v>6620</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-07-30 20:25:25</v>
+        <v>2026-08-03 12:26:10</v>
       </c>
       <c r="D20" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B21">
-        <v>6609</v>
+        <v>6620</v>
       </c>
       <c r="C21" t="str">
-        <v>2026-07-30 21:03:47</v>
+        <v>2026-08-03 22:01:18</v>
       </c>
       <c r="D21" t="str">
         <v>SI</v>
@@ -702,7 +702,7 @@
         <v>6620</v>
       </c>
       <c r="C22" t="str">
-        <v>2026-07-30 18:24:36</v>
+        <v>2026-08-04 14:40:43</v>
       </c>
       <c r="D22" t="str">
         <v>NO</v>
@@ -716,7 +716,7 @@
         <v>6620</v>
       </c>
       <c r="C23" t="str">
-        <v>2026-07-30 18:24:36</v>
+        <v>2026-08-07 16:29:03</v>
       </c>
       <c r="D23" t="str">
         <v>NO</v>
@@ -724,16 +724,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B24">
-        <v>6620</v>
+        <v>6610</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-07-30 21:05:12</v>
+        <v>2026-08-03 09:43:08</v>
       </c>
       <c r="D24" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="25">
@@ -744,7 +744,7 @@
         <v>6610</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-07-30 20:14:12</v>
+        <v>2026-08-04 00:01:46</v>
       </c>
       <c r="D25" t="str">
         <v>SI</v>
@@ -758,21 +758,21 @@
         <v>6610</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-07-30 21:08:04</v>
+        <v>2026-08-04 16:31:07</v>
       </c>
       <c r="D26" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B27">
-        <v>6583</v>
+        <v>6610</v>
       </c>
       <c r="C27" t="str">
-        <v>2026-07-30 16:41:21</v>
+        <v>2026-08-07 17:30:59</v>
       </c>
       <c r="D27" t="str">
         <v>NO</v>
@@ -786,7 +786,7 @@
         <v>6583</v>
       </c>
       <c r="C28" t="str">
-        <v>2026-07-30 16:41:21</v>
+        <v>2026-08-03 12:12:32</v>
       </c>
       <c r="D28" t="str">
         <v>NO</v>
@@ -800,7 +800,7 @@
         <v>6583</v>
       </c>
       <c r="C29" t="str">
-        <v>2026-07-30 20:17:06</v>
+        <v>2026-08-03 21:31:40</v>
       </c>
       <c r="D29" t="str">
         <v>SI</v>
@@ -814,10 +814,10 @@
         <v>6583</v>
       </c>
       <c r="C30" t="str">
-        <v>2026-07-30 20:30:55</v>
+        <v>2026-08-04 11:36:09</v>
       </c>
       <c r="D30" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="31">
@@ -828,24 +828,24 @@
         <v>6583</v>
       </c>
       <c r="C31" t="str">
-        <v>2026-07-30 20:44:02</v>
+        <v>2026-08-04 15:43:39</v>
       </c>
       <c r="D31" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GLP DF6 RXDL-61 OPERACIONES</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B32">
-        <v>6600</v>
+        <v>6583</v>
       </c>
       <c r="C32" t="str">
-        <v>2026-07-30 19:14:36</v>
+        <v>2026-08-07 17:56:28</v>
       </c>
       <c r="D32" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="33">
@@ -856,10 +856,10 @@
         <v>6600</v>
       </c>
       <c r="C33" t="str">
-        <v>2026-07-30 19:14:36</v>
+        <v>2026-08-03 14:30:29</v>
       </c>
       <c r="D33" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="34">
@@ -870,7 +870,7 @@
         <v>6600</v>
       </c>
       <c r="C34" t="str">
-        <v>2026-07-31 14:36:05</v>
+        <v>2026-08-04 15:30:08</v>
       </c>
       <c r="D34" t="str">
         <v>NO</v>
@@ -878,13 +878,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GLP DF6 RXDL-61 OPERACIONES</v>
       </c>
       <c r="B35">
-        <v>6593</v>
+        <v>6600</v>
       </c>
       <c r="C35" t="str">
-        <v>2026-07-30 17:02:34</v>
+        <v>2026-08-07 18:18:28</v>
       </c>
       <c r="D35" t="str">
         <v>NO</v>
@@ -898,7 +898,7 @@
         <v>6593</v>
       </c>
       <c r="C36" t="str">
-        <v>2026-07-30 17:02:34</v>
+        <v>2026-08-03 12:22:44</v>
       </c>
       <c r="D36" t="str">
         <v>NO</v>
@@ -912,7 +912,7 @@
         <v>6593</v>
       </c>
       <c r="C37" t="str">
-        <v>2026-07-30 21:32:39</v>
+        <v>2026-08-03 22:25:40</v>
       </c>
       <c r="D37" t="str">
         <v>SI</v>
@@ -920,13 +920,13 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B38">
-        <v>6597</v>
+        <v>6593</v>
       </c>
       <c r="C38" t="str">
-        <v>2026-07-30 14:46:39</v>
+        <v>2026-08-04 15:36:41</v>
       </c>
       <c r="D38" t="str">
         <v>NO</v>
@@ -934,13 +934,13 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B39">
-        <v>6597</v>
+        <v>6593</v>
       </c>
       <c r="C39" t="str">
-        <v>2026-07-30 14:46:39</v>
+        <v>2026-08-07 15:59:52</v>
       </c>
       <c r="D39" t="str">
         <v>NO</v>
@@ -954,7 +954,7 @@
         <v>6597</v>
       </c>
       <c r="C40" t="str">
-        <v>2026-07-30 20:17:44</v>
+        <v>2026-08-03 04:19:39</v>
       </c>
       <c r="D40" t="str">
         <v>SI</v>
@@ -968,7 +968,7 @@
         <v>6597</v>
       </c>
       <c r="C41" t="str">
-        <v>2026-07-30 21:29:13</v>
+        <v>2026-08-03 23:22:08</v>
       </c>
       <c r="D41" t="str">
         <v>SI</v>
@@ -976,27 +976,27 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B42">
-        <v>6598</v>
+        <v>6597</v>
       </c>
       <c r="C42" t="str">
-        <v>2026-07-30 22:46:18</v>
+        <v>2026-08-04 15:18:53</v>
       </c>
       <c r="D42" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B43">
-        <v>6586</v>
+        <v>6597</v>
       </c>
       <c r="C43" t="str">
-        <v>2026-07-27 12:10:20</v>
+        <v>2026-08-07 17:58:03</v>
       </c>
       <c r="D43" t="str">
         <v>NO</v>
@@ -1004,13 +1004,13 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B44">
-        <v>6586</v>
+        <v>6598</v>
       </c>
       <c r="C44" t="str">
-        <v>2026-07-30 14:33:26</v>
+        <v>2026-08-03 11:39:20</v>
       </c>
       <c r="D44" t="str">
         <v>NO</v>
@@ -1018,27 +1018,27 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B45">
-        <v>6586</v>
+        <v>6598</v>
       </c>
       <c r="C45" t="str">
-        <v>2026-07-30 14:33:26</v>
+        <v>2026-08-03 21:36:03</v>
       </c>
       <c r="D45" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B46">
-        <v>6586</v>
+        <v>6598</v>
       </c>
       <c r="C46" t="str">
-        <v>2026-07-30 16:23:24</v>
+        <v>2026-08-04 11:32:35</v>
       </c>
       <c r="D46" t="str">
         <v>NO</v>
@@ -1046,30 +1046,30 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B47">
-        <v>6586</v>
+        <v>6598</v>
       </c>
       <c r="C47" t="str">
-        <v>2026-07-30 16:23:24</v>
+        <v>2026-08-04 20:58:14</v>
       </c>
       <c r="D47" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B48">
-        <v>6586</v>
+        <v>6598</v>
       </c>
       <c r="C48" t="str">
-        <v>2026-07-30 20:06:50</v>
+        <v>2026-08-07 17:53:01</v>
       </c>
       <c r="D48" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="49">
@@ -1080,10 +1080,10 @@
         <v>6586</v>
       </c>
       <c r="C49" t="str">
-        <v>2026-07-30 20:31:32</v>
+        <v>2026-08-03 12:02:56</v>
       </c>
       <c r="D49" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="50">
@@ -1094,21 +1094,21 @@
         <v>6586</v>
       </c>
       <c r="C50" t="str">
-        <v>2026-07-30 20:40:54</v>
+        <v>2026-08-04 12:02:40</v>
       </c>
       <c r="D50" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B51">
-        <v>6604</v>
+        <v>6586</v>
       </c>
       <c r="C51" t="str">
-        <v>2026-07-27 14:15:16</v>
+        <v>2026-08-04 15:30:32</v>
       </c>
       <c r="D51" t="str">
         <v>NO</v>
@@ -1116,13 +1116,13 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B52">
-        <v>6604</v>
+        <v>6586</v>
       </c>
       <c r="C52" t="str">
-        <v>2026-07-30 14:30:59</v>
+        <v>2026-08-07 15:37:09</v>
       </c>
       <c r="D52" t="str">
         <v>NO</v>
@@ -1136,7 +1136,7 @@
         <v>6604</v>
       </c>
       <c r="C53" t="str">
-        <v>2026-07-30 14:30:59</v>
+        <v>2026-08-03 12:56:45</v>
       </c>
       <c r="D53" t="str">
         <v>NO</v>
@@ -1150,10 +1150,10 @@
         <v>6604</v>
       </c>
       <c r="C54" t="str">
-        <v>2026-07-30 18:22:45</v>
+        <v>2026-08-03 21:37:44</v>
       </c>
       <c r="D54" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="55">
@@ -1164,7 +1164,7 @@
         <v>6604</v>
       </c>
       <c r="C55" t="str">
-        <v>2026-07-30 18:22:45</v>
+        <v>2026-08-04 18:12:37</v>
       </c>
       <c r="D55" t="str">
         <v>NO</v>
@@ -1172,16 +1172,16 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B56">
-        <v>6601</v>
+        <v>6604</v>
       </c>
       <c r="C56" t="str">
-        <v>2026-07-30 16:03:58</v>
+        <v>2026-08-07 20:17:02</v>
       </c>
       <c r="D56" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="57">
@@ -1192,7 +1192,7 @@
         <v>6601</v>
       </c>
       <c r="C57" t="str">
-        <v>2026-07-30 16:03:58</v>
+        <v>2026-08-03 13:00:25</v>
       </c>
       <c r="D57" t="str">
         <v>NO</v>
@@ -1206,7 +1206,7 @@
         <v>6601</v>
       </c>
       <c r="C58" t="str">
-        <v>2026-07-30 20:05:46</v>
+        <v>2026-08-03 21:43:44</v>
       </c>
       <c r="D58" t="str">
         <v>SI</v>
@@ -1220,7 +1220,7 @@
         <v>6601</v>
       </c>
       <c r="C59" t="str">
-        <v>2026-07-31 13:32:02</v>
+        <v>2026-08-04 18:10:16</v>
       </c>
       <c r="D59" t="str">
         <v>NO</v>
@@ -1228,16 +1228,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B60">
-        <v>6606</v>
+        <v>6601</v>
       </c>
       <c r="C60" t="str">
-        <v>2026-07-30 15:13:24</v>
+        <v>2026-08-07 20:10:35</v>
       </c>
       <c r="D60" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="61">
@@ -1248,10 +1248,10 @@
         <v>6606</v>
       </c>
       <c r="C61" t="str">
-        <v>2026-07-30 15:13:24</v>
+        <v>2026-08-03 04:11:21</v>
       </c>
       <c r="D61" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="62">
@@ -1262,10 +1262,10 @@
         <v>6606</v>
       </c>
       <c r="C62" t="str">
-        <v>2026-07-30 15:46:42</v>
+        <v>2026-08-03 21:31:58</v>
       </c>
       <c r="D62" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="63">
@@ -1276,7 +1276,7 @@
         <v>6606</v>
       </c>
       <c r="C63" t="str">
-        <v>2026-07-30 20:07:37</v>
+        <v>2026-08-03 22:04:14</v>
       </c>
       <c r="D63" t="str">
         <v>SI</v>
@@ -1290,24 +1290,24 @@
         <v>6606</v>
       </c>
       <c r="C64" t="str">
-        <v>2026-07-30 20:41:04</v>
+        <v>2026-08-04 15:59:57</v>
       </c>
       <c r="D64" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B65">
-        <v>6580</v>
+        <v>6606</v>
       </c>
       <c r="C65" t="str">
-        <v>2026-07-30 15:06:09</v>
+        <v>2026-08-07 20:30:53</v>
       </c>
       <c r="D65" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="66">
@@ -1318,7 +1318,7 @@
         <v>6580</v>
       </c>
       <c r="C66" t="str">
-        <v>2026-07-30 15:06:09</v>
+        <v>2026-08-03 13:11:36</v>
       </c>
       <c r="D66" t="str">
         <v>NO</v>
@@ -1332,7 +1332,7 @@
         <v>6580</v>
       </c>
       <c r="C67" t="str">
-        <v>2026-07-30 15:49:59</v>
+        <v>2026-08-04 12:11:08</v>
       </c>
       <c r="D67" t="str">
         <v>NO</v>
@@ -1346,10 +1346,10 @@
         <v>6580</v>
       </c>
       <c r="C68" t="str">
-        <v>2026-07-30 20:02:33</v>
+        <v>2026-08-04 15:49:21</v>
       </c>
       <c r="D68" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="69">
@@ -1360,7 +1360,7 @@
         <v>6580</v>
       </c>
       <c r="C69" t="str">
-        <v>2026-07-31 12:16:04</v>
+        <v>2026-08-07 15:38:15</v>
       </c>
       <c r="D69" t="str">
         <v>NO</v>
@@ -1374,7 +1374,7 @@
         <v>6594</v>
       </c>
       <c r="C70" t="str">
-        <v>2026-07-30 14:53:24</v>
+        <v>2026-08-03 12:19:44</v>
       </c>
       <c r="D70" t="str">
         <v>NO</v>
@@ -1388,7 +1388,7 @@
         <v>6594</v>
       </c>
       <c r="C71" t="str">
-        <v>2026-07-30 14:53:24</v>
+        <v>2026-08-04 12:35:47</v>
       </c>
       <c r="D71" t="str">
         <v>NO</v>
@@ -1402,7 +1402,7 @@
         <v>6594</v>
       </c>
       <c r="C72" t="str">
-        <v>2026-07-30 15:57:45</v>
+        <v>2026-08-04 15:18:55</v>
       </c>
       <c r="D72" t="str">
         <v>NO</v>
@@ -1416,7 +1416,7 @@
         <v>6594</v>
       </c>
       <c r="C73" t="str">
-        <v>2026-07-30 22:46:03</v>
+        <v>2026-08-07 19:45:54</v>
       </c>
       <c r="D73" t="str">
         <v>SI</v>
@@ -1430,7 +1430,7 @@
         <v>6605</v>
       </c>
       <c r="C74" t="str">
-        <v>2026-07-27 12:23:18</v>
+        <v>2026-08-03 12:11:14</v>
       </c>
       <c r="D74" t="str">
         <v>NO</v>
@@ -1444,10 +1444,10 @@
         <v>6605</v>
       </c>
       <c r="C75" t="str">
-        <v>2026-07-30 16:58:42</v>
+        <v>2026-08-03 21:44:27</v>
       </c>
       <c r="D75" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="76">
@@ -1458,24 +1458,24 @@
         <v>6605</v>
       </c>
       <c r="C76" t="str">
-        <v>2026-07-31 12:33:45</v>
+        <v>2026-08-04 21:41:25</v>
       </c>
       <c r="D76" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B77">
-        <v>6603</v>
+        <v>6605</v>
       </c>
       <c r="C77" t="str">
-        <v>2026-07-27 13:26:44</v>
+        <v>2026-08-07 21:57:15</v>
       </c>
       <c r="D77" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="78">
@@ -1486,7 +1486,7 @@
         <v>6603</v>
       </c>
       <c r="C78" t="str">
-        <v>2026-07-30 15:14:08</v>
+        <v>2026-08-03 15:41:55</v>
       </c>
       <c r="D78" t="str">
         <v>NO</v>
@@ -1500,7 +1500,7 @@
         <v>6603</v>
       </c>
       <c r="C79" t="str">
-        <v>2026-07-30 15:14:08</v>
+        <v>2026-08-04 13:14:32</v>
       </c>
       <c r="D79" t="str">
         <v>NO</v>
@@ -1514,7 +1514,7 @@
         <v>6603</v>
       </c>
       <c r="C80" t="str">
-        <v>2026-07-30 17:11:48</v>
+        <v>2026-08-04 15:53:51</v>
       </c>
       <c r="D80" t="str">
         <v>NO</v>
@@ -1528,10 +1528,10 @@
         <v>6603</v>
       </c>
       <c r="C81" t="str">
-        <v>2026-07-30 20:46:24</v>
+        <v>2026-08-07 15:22:53</v>
       </c>
       <c r="D81" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="82">
@@ -1542,7 +1542,7 @@
         <v>6607</v>
       </c>
       <c r="C82" t="str">
-        <v>2026-07-27 10:15:18</v>
+        <v>2026-08-03 10:22:12</v>
       </c>
       <c r="D82" t="str">
         <v>NO</v>
@@ -1556,10 +1556,10 @@
         <v>6607</v>
       </c>
       <c r="C83" t="str">
-        <v>2026-07-30 14:23:32</v>
+        <v>2026-08-03 22:05:15</v>
       </c>
       <c r="D83" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="84">
@@ -1570,7 +1570,7 @@
         <v>6607</v>
       </c>
       <c r="C84" t="str">
-        <v>2026-07-30 14:23:32</v>
+        <v>2026-08-04 17:05:27</v>
       </c>
       <c r="D84" t="str">
         <v>NO</v>
@@ -1584,10 +1584,10 @@
         <v>6607</v>
       </c>
       <c r="C85" t="str">
-        <v>2026-07-30 21:02:29</v>
+        <v>2026-08-07 16:25:27</v>
       </c>
       <c r="D85" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="86">
@@ -1598,7 +1598,7 @@
         <v>6602</v>
       </c>
       <c r="C86" t="str">
-        <v>2026-07-27 10:53:20</v>
+        <v>2026-08-03 10:59:15</v>
       </c>
       <c r="D86" t="str">
         <v>NO</v>
@@ -1612,10 +1612,10 @@
         <v>6602</v>
       </c>
       <c r="C87" t="str">
-        <v>2026-07-30 15:16:13</v>
+        <v>2026-08-03 22:21:40</v>
       </c>
       <c r="D87" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="88">
@@ -1626,7 +1626,7 @@
         <v>6602</v>
       </c>
       <c r="C88" t="str">
-        <v>2026-07-30 15:16:13</v>
+        <v>2026-08-04 17:14:50</v>
       </c>
       <c r="D88" t="str">
         <v>NO</v>
@@ -1640,7 +1640,7 @@
         <v>6602</v>
       </c>
       <c r="C89" t="str">
-        <v>2026-07-30 18:48:57</v>
+        <v>2026-08-07 16:27:55</v>
       </c>
       <c r="D89" t="str">
         <v>NO</v>
@@ -1648,16 +1648,16 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B90">
-        <v>6602</v>
+        <v>6612</v>
       </c>
       <c r="C90" t="str">
-        <v>2026-07-30 20:39:13</v>
+        <v>2026-08-03 11:54:46</v>
       </c>
       <c r="D90" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="91">
@@ -1668,10 +1668,10 @@
         <v>6612</v>
       </c>
       <c r="C91" t="str">
-        <v>2026-07-27 12:14:30</v>
+        <v>2026-08-03 22:23:08</v>
       </c>
       <c r="D91" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="92">
@@ -1682,7 +1682,7 @@
         <v>6612</v>
       </c>
       <c r="C92" t="str">
-        <v>2026-07-30 18:01:14</v>
+        <v>2026-08-04 15:20:25</v>
       </c>
       <c r="D92" t="str">
         <v>NO</v>
@@ -1696,7 +1696,7 @@
         <v>6612</v>
       </c>
       <c r="C93" t="str">
-        <v>2026-07-30 18:01:14</v>
+        <v>2026-08-07 15:39:42</v>
       </c>
       <c r="D93" t="str">
         <v>NO</v>
@@ -1704,13 +1704,13 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B94">
-        <v>6612</v>
+        <v>6599</v>
       </c>
       <c r="C94" t="str">
-        <v>2026-07-31 12:03:35</v>
+        <v>2026-08-03 11:56:13</v>
       </c>
       <c r="D94" t="str">
         <v>NO</v>
@@ -1724,10 +1724,10 @@
         <v>6599</v>
       </c>
       <c r="C95" t="str">
-        <v>2026-07-27 11:58:07</v>
+        <v>2026-08-03 21:57:20</v>
       </c>
       <c r="D95" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="96">
@@ -1738,7 +1738,7 @@
         <v>6599</v>
       </c>
       <c r="C96" t="str">
-        <v>2026-07-30 13:44:54</v>
+        <v>2026-08-04 15:59:30</v>
       </c>
       <c r="D96" t="str">
         <v>NO</v>
@@ -1752,7 +1752,7 @@
         <v>6599</v>
       </c>
       <c r="C97" t="str">
-        <v>2026-07-31 12:03:01</v>
+        <v>2026-08-07 16:16:03</v>
       </c>
       <c r="D97" t="str">
         <v>NO</v>
@@ -1760,16 +1760,16 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>GV FOSERO SJHW-18 V OLIVARES</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B98">
-        <v>6592</v>
+        <v>6621</v>
       </c>
       <c r="C98" t="str">
-        <v>2026-07-27 08:27:58</v>
+        <v>2026-08-05 20:54:37</v>
       </c>
       <c r="D98" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="99">
@@ -1780,38 +1780,38 @@
         <v>6592</v>
       </c>
       <c r="C99" t="str">
-        <v>2026-07-31 21:25:46</v>
+        <v>2026-08-03 08:17:28</v>
       </c>
       <c r="D99" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B100">
-        <v>6595</v>
+        <v>6592</v>
       </c>
       <c r="C100" t="str">
-        <v>2026-07-27 10:52:15</v>
+        <v>2026-08-05 21:17:52</v>
       </c>
       <c r="D100" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B101">
-        <v>6595</v>
+        <v>6592</v>
       </c>
       <c r="C101" t="str">
-        <v>2026-07-30 14:27:54</v>
+        <v>2026-08-07 21:43:53</v>
       </c>
       <c r="D101" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="102">
@@ -1822,7 +1822,7 @@
         <v>6595</v>
       </c>
       <c r="C102" t="str">
-        <v>2026-07-30 14:27:54</v>
+        <v>2026-08-03 10:36:54</v>
       </c>
       <c r="D102" t="str">
         <v>NO</v>
@@ -1836,10 +1836,10 @@
         <v>6595</v>
       </c>
       <c r="C103" t="str">
-        <v>2026-07-30 15:44:25</v>
+        <v>2026-08-03 22:58:27</v>
       </c>
       <c r="D103" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="104">
@@ -1850,7 +1850,7 @@
         <v>6595</v>
       </c>
       <c r="C104" t="str">
-        <v>2026-07-30 16:40:21</v>
+        <v>2026-08-04 15:28:23</v>
       </c>
       <c r="D104" t="str">
         <v>NO</v>
@@ -1864,7 +1864,7 @@
         <v>6595</v>
       </c>
       <c r="C105" t="str">
-        <v>2026-07-30 22:51:55</v>
+        <v>2026-08-07 19:49:21</v>
       </c>
       <c r="D105" t="str">
         <v>SI</v>
@@ -1878,7 +1878,7 @@
         <v>6585</v>
       </c>
       <c r="C106" t="str">
-        <v>2026-07-27 11:10:46</v>
+        <v>2026-08-03 11:08:27</v>
       </c>
       <c r="D106" t="str">
         <v>NO</v>
@@ -1892,10 +1892,10 @@
         <v>6585</v>
       </c>
       <c r="C107" t="str">
-        <v>2026-07-30 14:52:40</v>
+        <v>2026-08-03 23:10:16</v>
       </c>
       <c r="D107" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="108">
@@ -1906,7 +1906,7 @@
         <v>6585</v>
       </c>
       <c r="C108" t="str">
-        <v>2026-07-30 14:52:40</v>
+        <v>2026-08-04 16:01:44</v>
       </c>
       <c r="D108" t="str">
         <v>NO</v>
@@ -1920,7 +1920,7 @@
         <v>6585</v>
       </c>
       <c r="C109" t="str">
-        <v>2026-07-30 17:32:22</v>
+        <v>2026-08-07 15:44:31</v>
       </c>
       <c r="D109" t="str">
         <v>NO</v>
@@ -1928,13 +1928,13 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>GV SHDV-50 C CARDENAS</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B110">
-        <v>6585</v>
+        <v>6588</v>
       </c>
       <c r="C110" t="str">
-        <v>2026-07-30 21:08:18</v>
+        <v>2026-08-03 04:02:26</v>
       </c>
       <c r="D110" t="str">
         <v>SI</v>
@@ -1948,7 +1948,7 @@
         <v>6588</v>
       </c>
       <c r="C111" t="str">
-        <v>2026-07-27 04:03:27</v>
+        <v>2026-08-03 21:59:47</v>
       </c>
       <c r="D111" t="str">
         <v>SI</v>
@@ -1962,10 +1962,10 @@
         <v>6588</v>
       </c>
       <c r="C112" t="str">
-        <v>2026-07-30 15:34:31</v>
+        <v>2026-08-05 02:04:31</v>
       </c>
       <c r="D112" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="113">
@@ -1976,21 +1976,21 @@
         <v>6588</v>
       </c>
       <c r="C113" t="str">
-        <v>2026-07-30 15:34:31</v>
+        <v>2026-08-08 02:13:27</v>
       </c>
       <c r="D113" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B114">
-        <v>6588</v>
+        <v>6587</v>
       </c>
       <c r="C114" t="str">
-        <v>2026-07-30 18:10:13</v>
+        <v>2026-08-03 10:10:28</v>
       </c>
       <c r="D114" t="str">
         <v>NO</v>
@@ -1998,16 +1998,16 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B115">
-        <v>6588</v>
+        <v>6587</v>
       </c>
       <c r="C115" t="str">
-        <v>2026-07-30 20:38:08</v>
+        <v>2026-08-04 10:07:31</v>
       </c>
       <c r="D115" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="116">
@@ -2018,7 +2018,7 @@
         <v>6587</v>
       </c>
       <c r="C116" t="str">
-        <v>2026-07-27 11:02:26</v>
+        <v>2026-08-04 15:20:33</v>
       </c>
       <c r="D116" t="str">
         <v>NO</v>
@@ -2032,7 +2032,7 @@
         <v>6587</v>
       </c>
       <c r="C117" t="str">
-        <v>2026-07-30 14:25:06</v>
+        <v>2026-08-07 16:12:21</v>
       </c>
       <c r="D117" t="str">
         <v>NO</v>
@@ -2040,13 +2040,13 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B118">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C118" t="str">
-        <v>2026-07-30 14:25:06</v>
+        <v>2026-08-03 17:54:39</v>
       </c>
       <c r="D118" t="str">
         <v>NO</v>
@@ -2054,27 +2054,27 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B119">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C119" t="str">
-        <v>2026-07-30 16:40:20</v>
+        <v>2026-08-03 22:04:17</v>
       </c>
       <c r="D119" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B120">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C120" t="str">
-        <v>2026-07-30 16:40:20</v>
+        <v>2026-08-04 17:59:02</v>
       </c>
       <c r="D120" t="str">
         <v>NO</v>
@@ -2082,27 +2082,27 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B121">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C121" t="str">
-        <v>2026-07-31 01:53:32</v>
+        <v>2026-08-07 18:02:52</v>
       </c>
       <c r="D121" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B122">
-        <v>6582</v>
+        <v>6589</v>
       </c>
       <c r="C122" t="str">
-        <v>2026-07-30 15:14:24</v>
+        <v>2026-08-03 10:28:49</v>
       </c>
       <c r="D122" t="str">
         <v>NO</v>
@@ -2110,13 +2110,13 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B123">
-        <v>6582</v>
+        <v>6589</v>
       </c>
       <c r="C123" t="str">
-        <v>2026-07-30 15:14:24</v>
+        <v>2026-08-04 10:24:25</v>
       </c>
       <c r="D123" t="str">
         <v>NO</v>
@@ -2124,13 +2124,13 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B124">
-        <v>6582</v>
+        <v>6589</v>
       </c>
       <c r="C124" t="str">
-        <v>2026-07-30 16:24:49</v>
+        <v>2026-08-04 17:21:02</v>
       </c>
       <c r="D124" t="str">
         <v>NO</v>
@@ -2138,27 +2138,27 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B125">
-        <v>6582</v>
+        <v>6589</v>
       </c>
       <c r="C125" t="str">
-        <v>2026-07-30 20:17:33</v>
+        <v>2026-08-07 16:56:12</v>
       </c>
       <c r="D125" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B126">
-        <v>6582</v>
+        <v>6596</v>
       </c>
       <c r="C126" t="str">
-        <v>2026-07-30 21:09:05</v>
+        <v>2026-08-03 04:04:12</v>
       </c>
       <c r="D126" t="str">
         <v>SI</v>
@@ -2166,27 +2166,27 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B127">
-        <v>6589</v>
+        <v>6596</v>
       </c>
       <c r="C127" t="str">
-        <v>2026-07-27 10:26:43</v>
+        <v>2026-08-04 01:33:39</v>
       </c>
       <c r="D127" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B128">
-        <v>6589</v>
+        <v>6596</v>
       </c>
       <c r="C128" t="str">
-        <v>2026-07-30 14:22:07</v>
+        <v>2026-08-04 16:02:33</v>
       </c>
       <c r="D128" t="str">
         <v>NO</v>
@@ -2194,69 +2194,69 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B129">
-        <v>6589</v>
+        <v>6596</v>
       </c>
       <c r="C129" t="str">
-        <v>2026-07-30 14:22:07</v>
+        <v>2026-08-08 01:43:20</v>
       </c>
       <c r="D129" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B130">
-        <v>6589</v>
+        <v>6619</v>
       </c>
       <c r="C130" t="str">
-        <v>2026-07-30 17:32:30</v>
+        <v>2026-08-03 21:08:45</v>
       </c>
       <c r="D130" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B131">
-        <v>6589</v>
+        <v>6619</v>
       </c>
       <c r="C131" t="str">
-        <v>2026-07-30 17:32:30</v>
+        <v>2026-08-03 21:25:10</v>
       </c>
       <c r="D131" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B132">
-        <v>6589</v>
+        <v>6619</v>
       </c>
       <c r="C132" t="str">
-        <v>2026-07-30 21:26:02</v>
+        <v>2026-08-04 10:28:45</v>
       </c>
       <c r="D132" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B133">
-        <v>6596</v>
+        <v>6619</v>
       </c>
       <c r="C133" t="str">
-        <v>2026-07-27 10:15:01</v>
+        <v>2026-08-04 16:53:22</v>
       </c>
       <c r="D133" t="str">
         <v>NO</v>
@@ -2264,13 +2264,13 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B134">
-        <v>6596</v>
+        <v>6619</v>
       </c>
       <c r="C134" t="str">
-        <v>2026-07-30 18:00:47</v>
+        <v>2026-08-07 15:22:48</v>
       </c>
       <c r="D134" t="str">
         <v>NO</v>
@@ -2278,13 +2278,13 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>JAC  LYTS-17 G GALEA</v>
       </c>
       <c r="B135">
-        <v>6596</v>
+        <v>6614</v>
       </c>
       <c r="C135" t="str">
-        <v>2026-07-30 18:00:47</v>
+        <v>2026-08-03 09:55:55</v>
       </c>
       <c r="D135" t="str">
         <v>NO</v>
@@ -2292,13 +2292,13 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>JAC  LYTS-17 G GALEA</v>
       </c>
       <c r="B136">
-        <v>6596</v>
+        <v>6614</v>
       </c>
       <c r="C136" t="str">
-        <v>2026-07-31 01:24:05</v>
+        <v>2026-08-03 21:39:01</v>
       </c>
       <c r="D136" t="str">
         <v>SI</v>
@@ -2312,7 +2312,7 @@
         <v>6614</v>
       </c>
       <c r="C137" t="str">
-        <v>2026-07-30 15:16:30</v>
+        <v>2026-08-04 17:19:13</v>
       </c>
       <c r="D137" t="str">
         <v>NO</v>
@@ -2326,50 +2326,22 @@
         <v>6614</v>
       </c>
       <c r="C138" t="str">
-        <v>2026-07-30 15:16:30</v>
+        <v>2026-08-07 16:48:51</v>
       </c>
       <c r="D138" t="str">
         <v>NO</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="str">
-        <v>JAC  LYTS-17 G GALEA</v>
-      </c>
-      <c r="B139">
-        <v>6614</v>
-      </c>
-      <c r="C139" t="str">
-        <v>2026-07-30 16:55:36</v>
-      </c>
-      <c r="D139" t="str">
-        <v>NO</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="str">
-        <v>JAC  LYTS-17 G GALEA</v>
-      </c>
-      <c r="B140">
-        <v>6614</v>
-      </c>
-      <c r="C140" t="str">
-        <v>2026-07-30 21:58:25</v>
-      </c>
-      <c r="D140" t="str">
-        <v>SI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D140"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D138"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2387,69 +2359,69 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B2">
-        <v>6583</v>
+        <v>6606</v>
       </c>
       <c r="C2">
         <v>5</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B3">
-        <v>6586</v>
+        <v>6588</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B4">
-        <v>6609</v>
+        <v>6605</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GC TSVS-89 M AEDO</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B5">
-        <v>6610</v>
+        <v>6596</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GLP DF6 RXDL-61 OPERACIONES</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B6">
-        <v>6600</v>
+        <v>6609</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -2471,10 +2443,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B8">
-        <v>6606</v>
+        <v>6598</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -2485,13 +2457,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B9">
-        <v>6588</v>
+        <v>6604</v>
       </c>
       <c r="C9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -2499,13 +2471,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B10">
-        <v>6582</v>
+        <v>6601</v>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10">
         <v>2</v>
@@ -2513,55 +2485,55 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>DONGFENG DF6 SRSR-97</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B11">
-        <v>6618</v>
+        <v>6592</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GV PEUGEOT THJY-73 J PONCE</v>
       </c>
       <c r="B12">
-        <v>6616</v>
+        <v>6595</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GC RXDL-59 OPERACIONES</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B13">
-        <v>6581</v>
+        <v>6619</v>
       </c>
       <c r="C13">
+        <v>5</v>
+      </c>
+      <c r="D13">
         <v>2</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>DONGFENG DF6 SRSR-97</v>
       </c>
       <c r="B14">
-        <v>6608</v>
+        <v>6618</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -2569,13 +2541,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B15">
-        <v>6620</v>
+        <v>6617</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -2583,13 +2555,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GC MAXUS PKFF-65 G VICENCIO</v>
       </c>
       <c r="B16">
-        <v>6593</v>
+        <v>6616</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -2597,13 +2569,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GC TM5-RXXG-13 D SILVA</v>
       </c>
       <c r="B17">
-        <v>6598</v>
+        <v>6608</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -2611,10 +2583,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B18">
-        <v>6601</v>
+        <v>6620</v>
       </c>
       <c r="C18">
         <v>4</v>
@@ -2625,13 +2597,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B19">
-        <v>6580</v>
+        <v>6610</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2639,13 +2611,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B20">
-        <v>6594</v>
+        <v>6583</v>
       </c>
       <c r="C20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2653,13 +2625,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B21">
-        <v>6603</v>
+        <v>6593</v>
       </c>
       <c r="C21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -2667,10 +2639,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GP DONGFENG DF6-RXDL-60</v>
+        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
       </c>
       <c r="B22">
-        <v>6607</v>
+        <v>6594</v>
       </c>
       <c r="C22">
         <v>4</v>
@@ -2681,13 +2653,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP DONGFENG DF6-RXDL-60</v>
       </c>
       <c r="B23">
-        <v>6602</v>
+        <v>6607</v>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2695,13 +2667,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GV FOSERO SJHW-18 V OLIVARES</v>
+        <v>GP FOTON G7 TSVS-96</v>
       </c>
       <c r="B24">
-        <v>6592</v>
+        <v>6602</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2709,13 +2681,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B25">
-        <v>6595</v>
+        <v>6612</v>
       </c>
       <c r="C25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -2723,13 +2695,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GV SHDV-50 C CARDENAS</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B26">
-        <v>6585</v>
+        <v>6599</v>
       </c>
       <c r="C26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -2737,13 +2709,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B27">
-        <v>6587</v>
+        <v>6621</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2751,13 +2723,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV SHDV-50 C CARDENAS</v>
       </c>
       <c r="B28">
-        <v>6589</v>
+        <v>6585</v>
       </c>
       <c r="C28">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -2765,10 +2737,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B29">
-        <v>6596</v>
+        <v>6582</v>
       </c>
       <c r="C29">
         <v>4</v>
@@ -2793,13 +2765,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GC MAXUS PCRF-25 TERRENO</v>
+        <v>GLP DF6 RXDL-61 OPERACIONES</v>
       </c>
       <c r="B31">
-        <v>6617</v>
+        <v>6600</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -2807,13 +2779,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B32">
-        <v>6604</v>
+        <v>6586</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -2821,13 +2793,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>GP -SHLC-76 F SEPULVEDA</v>
+        <v>GLP SSZD-71  J VALLEJOS</v>
       </c>
       <c r="B33">
-        <v>6605</v>
+        <v>6580</v>
       </c>
       <c r="C33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -2835,10 +2807,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GP CHANGAN RRDF-75 L LOBOS</v>
       </c>
       <c r="B34">
-        <v>6612</v>
+        <v>6603</v>
       </c>
       <c r="C34">
         <v>4</v>
@@ -2849,21 +2821,35 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>GP TM5 TSDK-95 L MUNOZ</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B35">
-        <v>6599</v>
+        <v>6587</v>
       </c>
       <c r="C35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
+      </c>
+      <c r="B36">
+        <v>6589</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-08-17 → 2026-08-23
</commit_message>
<xml_diff>
--- a/latest-events.xlsx
+++ b/latest-events.xlsx
@@ -422,7 +422,7 @@
         <v>6618</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-10 09:52:36</v>
+        <v>2026-08-17 09:11:08</v>
       </c>
       <c r="D2" t="str">
         <v>NO</v>
@@ -436,10 +436,10 @@
         <v>6617</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-10 05:20:18</v>
+        <v>2026-08-18 12:12:46</v>
       </c>
       <c r="D3" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="4">
@@ -450,35 +450,35 @@
         <v>6616</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-10 22:30:15</v>
+        <v>2026-08-17 14:13:16</v>
       </c>
       <c r="D4" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>GC RXDL-59 OPERACIONES</v>
       </c>
       <c r="B5">
-        <v>6608</v>
+        <v>6581</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-08-10 11:21:35</v>
+        <v>2026-08-19 19:04:39</v>
       </c>
       <c r="D5" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GC TM5-RXXG-13 D SILVA</v>
       </c>
       <c r="B6">
-        <v>6609</v>
+        <v>6608</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-08-10 11:17:09</v>
+        <v>2026-08-17 10:35:53</v>
       </c>
       <c r="D6" t="str">
         <v>NO</v>
@@ -486,13 +486,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B7">
-        <v>6620</v>
+        <v>6609</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-08-10 12:22:31</v>
+        <v>2026-08-17 11:18:30</v>
       </c>
       <c r="D7" t="str">
         <v>NO</v>
@@ -500,13 +500,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GC TSVS-89 M AEDO</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B8">
-        <v>6610</v>
+        <v>6620</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-08-10 09:46:18</v>
+        <v>2026-08-17 11:22:23</v>
       </c>
       <c r="D8" t="str">
         <v>NO</v>
@@ -514,13 +514,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B9">
-        <v>6583</v>
+        <v>6610</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-08-10 12:16:12</v>
+        <v>2026-08-17 09:48:32</v>
       </c>
       <c r="D9" t="str">
         <v>NO</v>
@@ -528,13 +528,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B10">
-        <v>6593</v>
+        <v>6583</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-08-10 12:33:50</v>
+        <v>2026-08-17 13:48:17</v>
       </c>
       <c r="D10" t="str">
         <v>NO</v>
@@ -542,41 +542,41 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B11">
-        <v>6597</v>
+        <v>6593</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-08-10 04:29:24</v>
+        <v>2026-08-17 12:31:16</v>
       </c>
       <c r="D11" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B12">
-        <v>6598</v>
+        <v>6597</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-08-10 11:41:26</v>
+        <v>2026-08-17 04:29:03</v>
       </c>
       <c r="D12" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B13">
-        <v>6586</v>
+        <v>6598</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-08-10 11:56:55</v>
+        <v>2026-08-17 11:36:50</v>
       </c>
       <c r="D13" t="str">
         <v>NO</v>
@@ -584,27 +584,27 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B14">
-        <v>6604</v>
+        <v>6586</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-08-10 20:05:38</v>
+        <v>2026-08-17 12:06:31</v>
       </c>
       <c r="D14" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B15">
-        <v>6601</v>
+        <v>6604</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-08-10 12:35:44</v>
+        <v>2026-08-17 13:49:40</v>
       </c>
       <c r="D15" t="str">
         <v>NO</v>
@@ -612,41 +612,41 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B16">
-        <v>6606</v>
+        <v>6601</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-08-10 05:38:25</v>
+        <v>2026-08-17 13:45:10</v>
       </c>
       <c r="D16" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B17">
-        <v>6580</v>
+        <v>6606</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-08-10 12:17:45</v>
+        <v>2026-08-17 04:50:09</v>
       </c>
       <c r="D17" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
+        <v>GLP SSZD-71  J VALLEJOS</v>
       </c>
       <c r="B18">
-        <v>6594</v>
+        <v>6580</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-08-10 10:45:06</v>
+        <v>2026-08-17 12:07:12</v>
       </c>
       <c r="D18" t="str">
         <v>NO</v>
@@ -654,13 +654,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GP -SHLC-76 F SEPULVEDA</v>
+        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
       </c>
       <c r="B19">
-        <v>6605</v>
+        <v>6594</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-08-10 12:10:17</v>
+        <v>2026-08-17 17:45:26</v>
       </c>
       <c r="D19" t="str">
         <v>NO</v>
@@ -668,13 +668,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B20">
-        <v>6603</v>
+        <v>6605</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-08-10 12:53:09</v>
+        <v>2026-08-17 14:13:45</v>
       </c>
       <c r="D20" t="str">
         <v>NO</v>
@@ -682,13 +682,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GP DONGFENG DF6-RXDL-60</v>
+        <v>GP CHANGAN RRDF-75 L LOBOS</v>
       </c>
       <c r="B21">
-        <v>6607</v>
+        <v>6603</v>
       </c>
       <c r="C21" t="str">
-        <v>2026-08-10 09:23:43</v>
+        <v>2026-08-17 12:48:30</v>
       </c>
       <c r="D21" t="str">
         <v>NO</v>
@@ -696,13 +696,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP DONGFENG DF6-RXDL-60</v>
       </c>
       <c r="B22">
-        <v>6602</v>
+        <v>6607</v>
       </c>
       <c r="C22" t="str">
-        <v>2026-08-10 10:34:41</v>
+        <v>2026-08-17 10:14:58</v>
       </c>
       <c r="D22" t="str">
         <v>NO</v>
@@ -710,13 +710,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GP FOTON G7 TSVS-96</v>
       </c>
       <c r="B23">
-        <v>6612</v>
+        <v>6602</v>
       </c>
       <c r="C23" t="str">
-        <v>2026-08-10 12:08:15</v>
+        <v>2026-08-17 11:46:09</v>
       </c>
       <c r="D23" t="str">
         <v>NO</v>
@@ -724,13 +724,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GP TM5 TSDK-95 L MUNOZ</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B24">
-        <v>6599</v>
+        <v>6612</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-08-10 12:34:36</v>
+        <v>2026-08-17 12:25:12</v>
       </c>
       <c r="D24" t="str">
         <v>NO</v>
@@ -738,27 +738,27 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GV FORD BU-9781 V OLIVARES</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B25">
-        <v>6621</v>
+        <v>6599</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-08-10 21:37:05</v>
+        <v>2026-08-17 10:25:18</v>
       </c>
       <c r="D25" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GV FOSERO SJHW-18 V OLIVARES</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B26">
-        <v>6592</v>
+        <v>6621</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-08-10 08:23:42</v>
+        <v>2026-08-18 12:11:13</v>
       </c>
       <c r="D26" t="str">
         <v>NO</v>
@@ -766,13 +766,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B27">
-        <v>6595</v>
+        <v>6592</v>
       </c>
       <c r="C27" t="str">
-        <v>2026-08-10 12:53:39</v>
+        <v>2026-08-17 08:19:27</v>
       </c>
       <c r="D27" t="str">
         <v>NO</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GV SHDV-50 C CARDENAS</v>
+        <v>GV PEUGEOT THJY-73 J PONCE</v>
       </c>
       <c r="B28">
-        <v>6585</v>
+        <v>6595</v>
       </c>
       <c r="C28" t="str">
-        <v>2026-08-10 10:41:22</v>
+        <v>2026-08-17 10:56:09</v>
       </c>
       <c r="D28" t="str">
         <v>NO</v>
@@ -794,13 +794,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GV SHDV-50 C CARDENAS</v>
       </c>
       <c r="B29">
-        <v>6588</v>
+        <v>6585</v>
       </c>
       <c r="C29" t="str">
-        <v>2026-08-10 10:00:42</v>
+        <v>2026-08-17 11:21:52</v>
       </c>
       <c r="D29" t="str">
         <v>NO</v>
@@ -808,41 +808,41 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B30">
-        <v>6587</v>
+        <v>6588</v>
       </c>
       <c r="C30" t="str">
-        <v>2026-08-10 10:10:06</v>
+        <v>2026-08-17 19:22:51</v>
       </c>
       <c r="D30" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B31">
-        <v>6582</v>
+        <v>6587</v>
       </c>
       <c r="C31" t="str">
-        <v>2026-08-10 05:19:51</v>
+        <v>2026-08-17 11:31:01</v>
       </c>
       <c r="D31" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B32">
-        <v>6589</v>
+        <v>6582</v>
       </c>
       <c r="C32" t="str">
-        <v>2026-08-10 11:59:01</v>
+        <v>2026-08-17 11:53:13</v>
       </c>
       <c r="D32" t="str">
         <v>NO</v>
@@ -850,44 +850,44 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B33">
-        <v>6596</v>
+        <v>6589</v>
       </c>
       <c r="C33" t="str">
-        <v>2026-08-10 05:13:10</v>
+        <v>2026-08-17 11:53:44</v>
       </c>
       <c r="D33" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B34">
-        <v>6619</v>
+        <v>6596</v>
       </c>
       <c r="C34" t="str">
-        <v>2026-08-10 21:58:09</v>
+        <v>2026-08-17 18:06:27</v>
       </c>
       <c r="D34" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>JAC  LYTS-17 G GALEA</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B35">
-        <v>6614</v>
+        <v>6619</v>
       </c>
       <c r="C35" t="str">
-        <v>2026-08-10 09:53:58</v>
+        <v>2026-08-17 19:35:34</v>
       </c>
       <c r="D35" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
   </sheetData>
@@ -917,10 +917,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>GC MAXUS PCRF-25 TERRENO</v>
+        <v>GC RXDL-59 OPERACIONES</v>
       </c>
       <c r="B2">
-        <v>6617</v>
+        <v>6581</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -931,10 +931,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B3">
-        <v>6616</v>
+        <v>6597</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -945,10 +945,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B4">
-        <v>6597</v>
+        <v>6606</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -959,10 +959,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B5">
-        <v>6604</v>
+        <v>6588</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -973,10 +973,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B6">
-        <v>6606</v>
+        <v>6619</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -987,66 +987,66 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GV FORD BU-9781 V OLIVARES</v>
+        <v>DONGFENG DF6 SRSR-97</v>
       </c>
       <c r="B7">
-        <v>6621</v>
+        <v>6618</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B8">
-        <v>6582</v>
+        <v>6617</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GC MAXUS PKFF-65 G VICENCIO</v>
       </c>
       <c r="B9">
-        <v>6596</v>
+        <v>6616</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+        <v>GC TM5-RXXG-13 D SILVA</v>
       </c>
       <c r="B10">
-        <v>6619</v>
+        <v>6608</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>DONGFENG DF6 SRSR-97</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B11">
-        <v>6618</v>
+        <v>6609</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1057,10 +1057,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B12">
-        <v>6608</v>
+        <v>6620</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1071,10 +1071,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B13">
-        <v>6609</v>
+        <v>6610</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1085,10 +1085,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B14">
-        <v>6620</v>
+        <v>6583</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1099,10 +1099,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GC TSVS-89 M AEDO</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B15">
-        <v>6610</v>
+        <v>6593</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1113,10 +1113,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B16">
-        <v>6583</v>
+        <v>6598</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B17">
-        <v>6593</v>
+        <v>6586</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1141,10 +1141,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B18">
-        <v>6598</v>
+        <v>6604</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1155,10 +1155,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B19">
-        <v>6586</v>
+        <v>6601</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1169,10 +1169,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GLP SSZD-71  J VALLEJOS</v>
       </c>
       <c r="B20">
-        <v>6601</v>
+        <v>6580</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1183,10 +1183,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
       </c>
       <c r="B21">
-        <v>6580</v>
+        <v>6594</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1197,10 +1197,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B22">
-        <v>6594</v>
+        <v>6605</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1211,10 +1211,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GP -SHLC-76 F SEPULVEDA</v>
+        <v>GP CHANGAN RRDF-75 L LOBOS</v>
       </c>
       <c r="B23">
-        <v>6605</v>
+        <v>6603</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -1225,10 +1225,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GP DONGFENG DF6-RXDL-60</v>
       </c>
       <c r="B24">
-        <v>6603</v>
+        <v>6607</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1239,10 +1239,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GP DONGFENG DF6-RXDL-60</v>
+        <v>GP FOTON G7 TSVS-96</v>
       </c>
       <c r="B25">
-        <v>6607</v>
+        <v>6602</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1253,10 +1253,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B26">
-        <v>6602</v>
+        <v>6612</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1267,10 +1267,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B27">
-        <v>6612</v>
+        <v>6599</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1281,10 +1281,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GP TM5 TSDK-95 L MUNOZ</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B28">
-        <v>6599</v>
+        <v>6621</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1337,10 +1337,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B32">
-        <v>6588</v>
+        <v>6587</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1351,10 +1351,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B33">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1379,10 +1379,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>JAC  LYTS-17 G GALEA</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B35">
-        <v>6614</v>
+        <v>6596</v>
       </c>
       <c r="C35">
         <v>1</v>

</xml_diff>

<commit_message>
auto: reporte semana 2026-08-24 → 2026-08-30
</commit_message>
<xml_diff>
--- a/latest-events.xlsx
+++ b/latest-events.xlsx
@@ -422,7 +422,7 @@
         <v>6618</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-17 09:11:08</v>
+        <v>2026-08-24 09:52:37</v>
       </c>
       <c r="D2" t="str">
         <v>NO</v>
@@ -436,7 +436,7 @@
         <v>6617</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-18 12:12:46</v>
+        <v>2026-08-24 12:18:21</v>
       </c>
       <c r="D3" t="str">
         <v>NO</v>
@@ -450,7 +450,7 @@
         <v>6616</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-17 14:13:16</v>
+        <v>2026-08-24 09:46:56</v>
       </c>
       <c r="D4" t="str">
         <v>NO</v>
@@ -458,27 +458,27 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GC RXDL-59 OPERACIONES</v>
+        <v>GC TM5-RXXG-13 D SILVA</v>
       </c>
       <c r="B5">
-        <v>6581</v>
+        <v>6608</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-08-19 19:04:39</v>
+        <v>2026-08-24 10:22:58</v>
       </c>
       <c r="D5" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B6">
-        <v>6608</v>
+        <v>6609</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-08-17 10:35:53</v>
+        <v>2026-08-24 11:18:17</v>
       </c>
       <c r="D6" t="str">
         <v>NO</v>
@@ -486,13 +486,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B7">
-        <v>6609</v>
+        <v>6620</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-08-17 11:18:30</v>
+        <v>2026-08-24 11:23:41</v>
       </c>
       <c r="D7" t="str">
         <v>NO</v>
@@ -500,13 +500,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B8">
-        <v>6620</v>
+        <v>6610</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-08-17 11:22:23</v>
+        <v>2026-08-24 18:02:29</v>
       </c>
       <c r="D8" t="str">
         <v>NO</v>
@@ -514,13 +514,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GC TSVS-89 M AEDO</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B9">
-        <v>6610</v>
+        <v>6583</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-08-17 09:48:32</v>
+        <v>2026-08-24 15:49:00</v>
       </c>
       <c r="D9" t="str">
         <v>NO</v>
@@ -528,13 +528,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B10">
-        <v>6583</v>
+        <v>6593</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-08-17 13:48:17</v>
+        <v>2026-08-24 12:38:38</v>
       </c>
       <c r="D10" t="str">
         <v>NO</v>
@@ -542,41 +542,41 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B11">
-        <v>6593</v>
+        <v>6597</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-08-17 12:31:16</v>
+        <v>2026-08-24 06:52:18</v>
       </c>
       <c r="D11" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B12">
-        <v>6597</v>
+        <v>6598</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-08-17 04:29:03</v>
+        <v>2026-08-24 11:49:46</v>
       </c>
       <c r="D12" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B13">
-        <v>6598</v>
+        <v>6586</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-08-17 11:36:50</v>
+        <v>2026-08-24 12:02:22</v>
       </c>
       <c r="D13" t="str">
         <v>NO</v>
@@ -584,13 +584,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B14">
-        <v>6586</v>
+        <v>6604</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-08-17 12:06:31</v>
+        <v>2026-08-24 12:53:48</v>
       </c>
       <c r="D14" t="str">
         <v>NO</v>
@@ -598,13 +598,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B15">
-        <v>6604</v>
+        <v>6601</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-08-17 13:49:40</v>
+        <v>2026-08-24 13:31:21</v>
       </c>
       <c r="D15" t="str">
         <v>NO</v>
@@ -612,13 +612,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B16">
-        <v>6601</v>
+        <v>6606</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-08-17 13:45:10</v>
+        <v>2026-08-24 10:17:07</v>
       </c>
       <c r="D16" t="str">
         <v>NO</v>
@@ -626,27 +626,27 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>GLP SSZD-71  J VALLEJOS</v>
       </c>
       <c r="B17">
-        <v>6606</v>
+        <v>6580</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-08-17 04:50:09</v>
+        <v>2026-08-24 12:00:50</v>
       </c>
       <c r="D17" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
       </c>
       <c r="B18">
-        <v>6580</v>
+        <v>6594</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-08-17 12:07:12</v>
+        <v>2026-08-24 11:58:25</v>
       </c>
       <c r="D18" t="str">
         <v>NO</v>
@@ -654,13 +654,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B19">
-        <v>6594</v>
+        <v>6605</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-08-17 17:45:26</v>
+        <v>2026-08-24 12:37:53</v>
       </c>
       <c r="D19" t="str">
         <v>NO</v>
@@ -668,27 +668,27 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GP -SHLC-76 F SEPULVEDA</v>
+        <v>GP CHANGAN RRDF-75 L LOBOS</v>
       </c>
       <c r="B20">
-        <v>6605</v>
+        <v>6603</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-08-17 14:13:45</v>
+        <v>2026-08-24 06:02:10</v>
       </c>
       <c r="D20" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GP DONGFENG DF6-RXDL-60</v>
       </c>
       <c r="B21">
-        <v>6603</v>
+        <v>6607</v>
       </c>
       <c r="C21" t="str">
-        <v>2026-08-17 12:48:30</v>
+        <v>2026-08-24 10:14:42</v>
       </c>
       <c r="D21" t="str">
         <v>NO</v>
@@ -696,13 +696,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GP DONGFENG DF6-RXDL-60</v>
+        <v>GP FOTON G7 TSVS-96</v>
       </c>
       <c r="B22">
-        <v>6607</v>
+        <v>6602</v>
       </c>
       <c r="C22" t="str">
-        <v>2026-08-17 10:14:58</v>
+        <v>2026-08-24 10:52:38</v>
       </c>
       <c r="D22" t="str">
         <v>NO</v>
@@ -710,13 +710,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B23">
-        <v>6602</v>
+        <v>6612</v>
       </c>
       <c r="C23" t="str">
-        <v>2026-08-17 11:46:09</v>
+        <v>2026-08-24 10:48:32</v>
       </c>
       <c r="D23" t="str">
         <v>NO</v>
@@ -724,13 +724,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B24">
-        <v>6612</v>
+        <v>6599</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-08-17 12:25:12</v>
+        <v>2026-08-24 11:52:41</v>
       </c>
       <c r="D24" t="str">
         <v>NO</v>
@@ -738,13 +738,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GP TM5 TSDK-95 L MUNOZ</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B25">
-        <v>6599</v>
+        <v>6621</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-08-17 10:25:18</v>
+        <v>2026-08-25 12:12:37</v>
       </c>
       <c r="D25" t="str">
         <v>NO</v>
@@ -752,13 +752,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GV FORD BU-9781 V OLIVARES</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B26">
-        <v>6621</v>
+        <v>6592</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-08-18 12:11:13</v>
+        <v>2026-08-24 08:16:27</v>
       </c>
       <c r="D26" t="str">
         <v>NO</v>
@@ -766,13 +766,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GV FOSERO SJHW-18 V OLIVARES</v>
+        <v>GV PEUGEOT THJY-73 J PONCE</v>
       </c>
       <c r="B27">
-        <v>6592</v>
+        <v>6595</v>
       </c>
       <c r="C27" t="str">
-        <v>2026-08-17 08:19:27</v>
+        <v>2026-08-24 11:13:59</v>
       </c>
       <c r="D27" t="str">
         <v>NO</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GV SHDV-50 C CARDENAS</v>
       </c>
       <c r="B28">
-        <v>6595</v>
+        <v>6585</v>
       </c>
       <c r="C28" t="str">
-        <v>2026-08-17 10:56:09</v>
+        <v>2026-08-24 11:16:07</v>
       </c>
       <c r="D28" t="str">
         <v>NO</v>
@@ -794,13 +794,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GV SHDV-50 C CARDENAS</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B29">
-        <v>6585</v>
+        <v>6588</v>
       </c>
       <c r="C29" t="str">
-        <v>2026-08-17 11:21:52</v>
+        <v>2026-08-24 12:12:41</v>
       </c>
       <c r="D29" t="str">
         <v>NO</v>
@@ -808,27 +808,27 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B30">
-        <v>6588</v>
+        <v>6587</v>
       </c>
       <c r="C30" t="str">
-        <v>2026-08-17 19:22:51</v>
+        <v>2026-08-24 11:24:36</v>
       </c>
       <c r="D30" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B31">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C31" t="str">
-        <v>2026-08-17 11:31:01</v>
+        <v>2026-08-24 11:54:32</v>
       </c>
       <c r="D31" t="str">
         <v>NO</v>
@@ -836,13 +836,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B32">
-        <v>6582</v>
+        <v>6589</v>
       </c>
       <c r="C32" t="str">
-        <v>2026-08-17 11:53:13</v>
+        <v>2026-08-24 12:01:27</v>
       </c>
       <c r="D32" t="str">
         <v>NO</v>
@@ -850,13 +850,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B33">
-        <v>6589</v>
+        <v>6596</v>
       </c>
       <c r="C33" t="str">
-        <v>2026-08-17 11:53:44</v>
+        <v>2026-08-24 12:08:13</v>
       </c>
       <c r="D33" t="str">
         <v>NO</v>
@@ -864,13 +864,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B34">
-        <v>6596</v>
+        <v>6619</v>
       </c>
       <c r="C34" t="str">
-        <v>2026-08-17 18:06:27</v>
+        <v>2026-08-24 11:30:02</v>
       </c>
       <c r="D34" t="str">
         <v>NO</v>
@@ -878,13 +878,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+        <v>JAC  LYTS-17 G GALEA</v>
       </c>
       <c r="B35">
-        <v>6619</v>
+        <v>6614</v>
       </c>
       <c r="C35" t="str">
-        <v>2026-08-17 19:35:34</v>
+        <v>2026-08-26 19:53:11</v>
       </c>
       <c r="D35" t="str">
         <v>SI</v>
@@ -917,10 +917,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>GC RXDL-59 OPERACIONES</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B2">
-        <v>6581</v>
+        <v>6597</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -931,10 +931,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GP CHANGAN RRDF-75 L LOBOS</v>
       </c>
       <c r="B3">
-        <v>6597</v>
+        <v>6603</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -945,10 +945,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>JAC  LYTS-17 G GALEA</v>
       </c>
       <c r="B4">
-        <v>6606</v>
+        <v>6614</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -959,38 +959,38 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>DONGFENG DF6 SRSR-97</v>
       </c>
       <c r="B5">
-        <v>6588</v>
+        <v>6618</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B6">
-        <v>6619</v>
+        <v>6617</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>DONGFENG DF6 SRSR-97</v>
+        <v>GC MAXUS PKFF-65 G VICENCIO</v>
       </c>
       <c r="B7">
-        <v>6618</v>
+        <v>6616</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1001,10 +1001,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GC MAXUS PCRF-25 TERRENO</v>
+        <v>GC TM5-RXXG-13 D SILVA</v>
       </c>
       <c r="B8">
-        <v>6617</v>
+        <v>6608</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1015,10 +1015,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B9">
-        <v>6616</v>
+        <v>6609</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B10">
-        <v>6608</v>
+        <v>6620</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1043,10 +1043,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GC TSVS-89 M AEDO</v>
       </c>
       <c r="B11">
-        <v>6609</v>
+        <v>6610</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1057,10 +1057,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B12">
-        <v>6620</v>
+        <v>6583</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1071,10 +1071,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GC TSVS-89 M AEDO</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B13">
-        <v>6610</v>
+        <v>6593</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1085,10 +1085,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B14">
-        <v>6583</v>
+        <v>6598</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1099,10 +1099,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B15">
-        <v>6593</v>
+        <v>6586</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1113,10 +1113,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B16">
-        <v>6598</v>
+        <v>6604</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B17">
-        <v>6586</v>
+        <v>6601</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1141,10 +1141,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B18">
-        <v>6604</v>
+        <v>6606</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1155,10 +1155,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GLP SSZD-71  J VALLEJOS</v>
       </c>
       <c r="B19">
-        <v>6601</v>
+        <v>6580</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1169,10 +1169,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
       </c>
       <c r="B20">
-        <v>6580</v>
+        <v>6594</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1183,10 +1183,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B21">
-        <v>6594</v>
+        <v>6605</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1197,10 +1197,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GP -SHLC-76 F SEPULVEDA</v>
+        <v>GP DONGFENG DF6-RXDL-60</v>
       </c>
       <c r="B22">
-        <v>6605</v>
+        <v>6607</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1211,10 +1211,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GP FOTON G7 TSVS-96</v>
       </c>
       <c r="B23">
-        <v>6603</v>
+        <v>6602</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -1225,10 +1225,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GP DONGFENG DF6-RXDL-60</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B24">
-        <v>6607</v>
+        <v>6612</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1239,10 +1239,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B25">
-        <v>6602</v>
+        <v>6599</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1253,10 +1253,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B26">
-        <v>6612</v>
+        <v>6621</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1267,10 +1267,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GP TM5 TSDK-95 L MUNOZ</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B27">
-        <v>6599</v>
+        <v>6592</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1281,10 +1281,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GV FORD BU-9781 V OLIVARES</v>
+        <v>GV PEUGEOT THJY-73 J PONCE</v>
       </c>
       <c r="B28">
-        <v>6621</v>
+        <v>6595</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1295,10 +1295,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GV FOSERO SJHW-18 V OLIVARES</v>
+        <v>GV SHDV-50 C CARDENAS</v>
       </c>
       <c r="B29">
-        <v>6592</v>
+        <v>6585</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1309,10 +1309,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B30">
-        <v>6595</v>
+        <v>6588</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1323,10 +1323,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GV SHDV-50 C CARDENAS</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B31">
-        <v>6585</v>
+        <v>6587</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1337,10 +1337,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B32">
-        <v>6587</v>
+        <v>6582</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1351,10 +1351,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B33">
-        <v>6582</v>
+        <v>6589</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B34">
-        <v>6589</v>
+        <v>6596</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -1379,10 +1379,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
       </c>
       <c r="B35">
-        <v>6596</v>
+        <v>6619</v>
       </c>
       <c r="C35">
         <v>1</v>

</xml_diff>